<commit_message>
almost ready for fabrication
</commit_message>
<xml_diff>
--- a/PCB/bom/Attendance_Management_System_BOM_DigiKey.xlsx
+++ b/PCB/bom/Attendance_Management_System_BOM_DigiKey.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="341">
   <si>
     <t xml:space="preserve">How to order</t>
   </si>
@@ -48,7 +48,7 @@
     <t xml:space="preserve">U5, NFC reader: ST25R3916-AQWT is out of stock at Digi-Key (the ST25R3916B is not due until 2028). The in-stock ST25R3917-AQWT is pin-compatible but has no capacitive-sensor wake-up, no automatic antenna tuning and no card emulation. It works for this reader if the firmware uses inductive wake-up and J5/J6 stay unconnected. Set U5 "Use alternate" = Y to order it, or source the ST25R3916 elsewhere.</t>
   </si>
   <si>
-    <t xml:space="preserve">Y2 + C6/C7, 32.768 kHz: no 4 pF-load 3.2x1.5 mm crystal is stocked, so Y2 is a 6 pF part and C6/C7 default to the 8.2 pF alternate. Update C6/C7 to 8.2p in the schematic so the design matches what you build.</t>
+    <t xml:space="preserve">Y2 + C6/C7, 32.768 kHz: no 4 pF-load 3.2x1.5 mm crystal is stocked, so Y2 is a 6 pF part and C6/C7 were changed to 8.2 pF in the schematic (2026-09-26).</t>
   </si>
   <si>
     <t xml:space="preserve">R6, charge current: 1 kΩ sets 1 A, above the 500 mA a USB-C sink with 5.1 kΩ CC resistors may draw. The 2 kΩ alternate gives 500 mA.</t>
@@ -252,16 +252,10 @@
     <t xml:space="preserve">C6,C7</t>
   </si>
   <si>
-    <t xml:space="preserve">4.3p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor, ceramic, 4.3 pF 50 V C0G ±0.25 pF (LSE load caps)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C0805C439C5GACTU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">399-C0805C439C5GACTUCT-ND</t>
+    <t xml:space="preserve">8.2p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitor, ceramic, 8.2 pF 50 V C0G ±0.25 pF (LSE load caps)</t>
   </si>
   <si>
     <t xml:space="preserve">C0805C829C5GACTU</t>
@@ -270,7 +264,7 @@
     <t xml:space="preserve">399-C0805C829C5GACTUCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">ALTERNATE ON by default: Y2 below has CL = 6 pF (no 4 pF 3.2x1.5 mm crystal is stocked), which needs 8.2 pF load caps: CL = C/2 + ~2 pF stray. With 4.3 pF the RTC runs ~70 ppm fast (~6 s/day). Change C6/C7 to 8.2p in the schematic.</t>
+    <t xml:space="preserve">Y2 has CL = 6 pF (no 4 pF 3.2x1.5 mm crystal is stocked), which needs 8.2 pF load caps: CL = C/2 + ~2 pF stray. Changed from 4.3p in the schematic on 2026-09-26.</t>
   </si>
   <si>
     <t xml:space="preserve">C9,C10</t>
@@ -990,7 +984,7 @@
     <t xml:space="preserve">535-11937-1-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">Lowest-CL 3.2x1.5 mm crystal in stock (no 4 pF part). Needs 8.2 pF load caps (C6/C7 alternate). Check the land pattern against the EuroQuartz EQ161 footprint.</t>
+    <t xml:space="preserve">Lowest-CL 3.2x1.5 mm crystal in stock (no 4 pF part). Needs the 8.2 pF load caps C6/C7. Check the land pattern against the EuroQuartz EQ161 footprint.</t>
   </si>
   <si>
     <t xml:space="preserve">AE3</t>
@@ -1926,15 +1920,15 @@
         <v>15</v>
       </c>
       <c r="V8" s="8" t="str">
-        <f aca="false">IF(M8="Y",N8,G8)</f>
+        <f aca="false">IF(M8="Y",N8,G8)&amp;""</f>
         <v>Samsung Electro-Mechanics</v>
       </c>
       <c r="W8" s="8" t="str">
-        <f aca="false">IF(M8="Y",O8,H8)</f>
+        <f aca="false">IF(M8="Y",O8,H8)&amp;""</f>
         <v>CL21B104KBCNNNC</v>
       </c>
       <c r="X8" s="8" t="str">
-        <f aca="false">IF(M8="Y",P8,I8)</f>
+        <f aca="false">IF(M8="Y",P8,I8)&amp;""</f>
         <v>1276-1003-1-ND</v>
       </c>
       <c r="Y8" s="12" t="n">
@@ -2005,15 +1999,15 @@
         <v>4</v>
       </c>
       <c r="V9" s="13" t="str">
-        <f aca="false">IF(M9="Y",N9,G9)</f>
+        <f aca="false">IF(M9="Y",N9,G9)&amp;""</f>
         <v>Samsung Electro-Mechanics</v>
       </c>
       <c r="W9" s="13" t="str">
-        <f aca="false">IF(M9="Y",O9,H9)</f>
+        <f aca="false">IF(M9="Y",O9,H9)&amp;""</f>
         <v>CL21A475KACLRNC</v>
       </c>
       <c r="X9" s="13" t="str">
-        <f aca="false">IF(M9="Y",P9,I9)</f>
+        <f aca="false">IF(M9="Y",P9,I9)&amp;""</f>
         <v>1276-2415-1-ND</v>
       </c>
       <c r="Y9" s="16" t="n">
@@ -2084,15 +2078,15 @@
         <v>3</v>
       </c>
       <c r="V10" s="8" t="str">
-        <f aca="false">IF(M10="Y",N10,G10)</f>
+        <f aca="false">IF(M10="Y",N10,G10)&amp;""</f>
         <v>Samsung Electro-Mechanics</v>
       </c>
       <c r="W10" s="8" t="str">
-        <f aca="false">IF(M10="Y",O10,H10)</f>
+        <f aca="false">IF(M10="Y",O10,H10)&amp;""</f>
         <v>CL21B103KBANNNC</v>
       </c>
       <c r="X10" s="8" t="str">
-        <f aca="false">IF(M10="Y",P10,I10)</f>
+        <f aca="false">IF(M10="Y",P10,I10)&amp;""</f>
         <v>1276-1015-1-ND</v>
       </c>
       <c r="Y10" s="12" t="n">
@@ -2161,15 +2155,15 @@
         <v>4</v>
       </c>
       <c r="V11" s="13" t="str">
-        <f aca="false">IF(M11="Y",N11,G11)</f>
+        <f aca="false">IF(M11="Y",N11,G11)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W11" s="13" t="str">
-        <f aca="false">IF(M11="Y",O11,H11)</f>
+        <f aca="false">IF(M11="Y",O11,H11)&amp;""</f>
         <v>C0805C105K3RACTU</v>
       </c>
       <c r="X11" s="13" t="str">
-        <f aca="false">IF(M11="Y",P11,I11)</f>
+        <f aca="false">IF(M11="Y",P11,I11)&amp;""</f>
         <v>399-C0805C105K3RACTUCT-ND</v>
       </c>
       <c r="Y11" s="16" t="n">
@@ -2184,7 +2178,7 @@
         <v>open</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="n">
         <v>5</v>
       </c>
@@ -2213,32 +2207,22 @@
         <v>78</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>1703</v>
+        <v>3279</v>
       </c>
       <c r="K12" s="10" t="n">
-        <v>0.326</v>
+        <v>0.372</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>10</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="N12" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="O12" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="P12" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q12" s="9" t="n">
-        <v>3279</v>
-      </c>
-      <c r="R12" s="10" t="n">
-        <v>0.372</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="10"/>
       <c r="S12" s="11" t="s">
         <v>54</v>
       </c>
@@ -2250,15 +2234,15 @@
         <v>4</v>
       </c>
       <c r="V12" s="8" t="str">
-        <f aca="false">IF(M12="Y",N12,G12)</f>
+        <f aca="false">IF(M12="Y",N12,G12)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W12" s="8" t="str">
-        <f aca="false">IF(M12="Y",O12,H12)</f>
+        <f aca="false">IF(M12="Y",O12,H12)&amp;""</f>
         <v>C0805C829C5GACTU</v>
       </c>
       <c r="X12" s="8" t="str">
-        <f aca="false">IF(M12="Y",P12,I12)</f>
+        <f aca="false">IF(M12="Y",P12,I12)&amp;""</f>
         <v>399-C0805C829C5GACTUCT-ND</v>
       </c>
       <c r="Y12" s="12" t="n">
@@ -2266,7 +2250,7 @@
         <v>1.488</v>
       </c>
       <c r="Z12" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="AA12" s="8" t="str">
         <f aca="false">IF(W12="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W12,"open"))</f>
@@ -2278,16 +2262,16 @@
         <v>6</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>49</v>
@@ -2296,10 +2280,10 @@
         <v>70</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J13" s="14" t="n">
         <v>28868</v>
@@ -2329,15 +2313,15 @@
         <v>4</v>
       </c>
       <c r="V13" s="13" t="str">
-        <f aca="false">IF(M13="Y",N13,G13)</f>
+        <f aca="false">IF(M13="Y",N13,G13)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W13" s="13" t="str">
-        <f aca="false">IF(M13="Y",O13,H13)</f>
+        <f aca="false">IF(M13="Y",O13,H13)&amp;""</f>
         <v>C0805C150J5GACTU</v>
       </c>
       <c r="X13" s="13" t="str">
-        <f aca="false">IF(M13="Y",P13,I13)</f>
+        <f aca="false">IF(M13="Y",P13,I13)&amp;""</f>
         <v>399-C0805C150J5GACTUCT-ND</v>
       </c>
       <c r="Y13" s="16" t="n">
@@ -2345,7 +2329,7 @@
         <v>0.64</v>
       </c>
       <c r="Z13" s="13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AA13" s="13" t="str">
         <f aca="false">IF(W13="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W13,"open"))</f>
@@ -2357,16 +2341,16 @@
         <v>7</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>4</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>49</v>
@@ -2375,10 +2359,10 @@
         <v>70</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J14" s="9" t="n">
         <v>62894</v>
@@ -2408,15 +2392,15 @@
         <v>6</v>
       </c>
       <c r="V14" s="8" t="str">
-        <f aca="false">IF(M14="Y",N14,G14)</f>
+        <f aca="false">IF(M14="Y",N14,G14)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W14" s="8" t="str">
-        <f aca="false">IF(M14="Y",O14,H14)</f>
+        <f aca="false">IF(M14="Y",O14,H14)&amp;""</f>
         <v>C0805C151J5GACTU</v>
       </c>
       <c r="X14" s="8" t="str">
-        <f aca="false">IF(M14="Y",P14,I14)</f>
+        <f aca="false">IF(M14="Y",P14,I14)&amp;""</f>
         <v>399-C0805C151J5GACTUCT-ND</v>
       </c>
       <c r="Y14" s="12" t="n">
@@ -2424,7 +2408,7 @@
         <v>0.48</v>
       </c>
       <c r="Z14" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AA14" s="8" t="str">
         <f aca="false">IF(W14="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W14,"open"))</f>
@@ -2436,16 +2420,16 @@
         <v>8</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>49</v>
@@ -2454,10 +2438,10 @@
         <v>70</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J15" s="14" t="n">
         <v>215055</v>
@@ -2487,15 +2471,15 @@
         <v>4</v>
       </c>
       <c r="V15" s="13" t="str">
-        <f aca="false">IF(M15="Y",N15,G15)</f>
+        <f aca="false">IF(M15="Y",N15,G15)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W15" s="13" t="str">
-        <f aca="false">IF(M15="Y",O15,H15)</f>
+        <f aca="false">IF(M15="Y",O15,H15)&amp;""</f>
         <v>C0805C100J5GACTU</v>
       </c>
       <c r="X15" s="13" t="str">
-        <f aca="false">IF(M15="Y",P15,I15)</f>
+        <f aca="false">IF(M15="Y",P15,I15)&amp;""</f>
         <v>399-C0805C100J5GAC7800CT-ND</v>
       </c>
       <c r="Y15" s="16" t="n">
@@ -2503,7 +2487,7 @@
         <v>0.304</v>
       </c>
       <c r="Z15" s="13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="AA15" s="13" t="str">
         <f aca="false">IF(W15="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W15,"open"))</f>
@@ -2515,16 +2499,16 @@
         <v>9</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>49</v>
@@ -2533,10 +2517,10 @@
         <v>70</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J16" s="9" t="n">
         <v>20555</v>
@@ -2566,15 +2550,15 @@
         <v>6</v>
       </c>
       <c r="V16" s="8" t="str">
-        <f aca="false">IF(M16="Y",N16,G16)</f>
+        <f aca="false">IF(M16="Y",N16,G16)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W16" s="8" t="str">
-        <f aca="false">IF(M16="Y",O16,H16)</f>
+        <f aca="false">IF(M16="Y",O16,H16)&amp;""</f>
         <v>C0805C680J5GACTU</v>
       </c>
       <c r="X16" s="8" t="str">
-        <f aca="false">IF(M16="Y",P16,I16)</f>
+        <f aca="false">IF(M16="Y",P16,I16)&amp;""</f>
         <v>399-C0805C680J5GACTUCT-ND</v>
       </c>
       <c r="Y16" s="12" t="n">
@@ -2582,7 +2566,7 @@
         <v>0.636</v>
       </c>
       <c r="Z16" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="AA16" s="8" t="str">
         <f aca="false">IF(W16="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W16,"open"))</f>
@@ -2594,16 +2578,16 @@
         <v>10</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>49</v>
@@ -2612,10 +2596,10 @@
         <v>70</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J17" s="14" t="n">
         <v>147889</v>
@@ -2645,15 +2629,15 @@
         <v>6</v>
       </c>
       <c r="V17" s="13" t="str">
-        <f aca="false">IF(M17="Y",N17,G17)</f>
+        <f aca="false">IF(M17="Y",N17,G17)&amp;""</f>
         <v>KEMET</v>
       </c>
       <c r="W17" s="13" t="str">
-        <f aca="false">IF(M17="Y",O17,H17)</f>
+        <f aca="false">IF(M17="Y",O17,H17)&amp;""</f>
         <v>C0805C271J5GACTU</v>
       </c>
       <c r="X17" s="13" t="str">
-        <f aca="false">IF(M17="Y",P17,I17)</f>
+        <f aca="false">IF(M17="Y",P17,I17)&amp;""</f>
         <v>399-C0805C271J5GACTUCT-ND</v>
       </c>
       <c r="Y17" s="16" t="n">
@@ -2661,7 +2645,7 @@
         <v>1.296</v>
       </c>
       <c r="Z17" s="13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA17" s="13" t="str">
         <f aca="false">IF(W17="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W17,"open"))</f>
@@ -2673,16 +2657,16 @@
         <v>11</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>49</v>
@@ -2691,10 +2675,10 @@
         <v>50</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J18" s="9" t="n">
         <v>178</v>
@@ -2709,13 +2693,13 @@
         <v>53</v>
       </c>
       <c r="N18" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="P18" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="O18" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="P18" s="8" t="s">
-        <v>119</v>
       </c>
       <c r="Q18" s="9" t="n">
         <v>5598</v>
@@ -2734,15 +2718,15 @@
         <v>4</v>
       </c>
       <c r="V18" s="8" t="str">
-        <f aca="false">IF(M18="Y",N18,G18)</f>
+        <f aca="false">IF(M18="Y",N18,G18)&amp;""</f>
         <v>Samsung Electro-Mechanics</v>
       </c>
       <c r="W18" s="8" t="str">
-        <f aca="false">IF(M18="Y",O18,H18)</f>
+        <f aca="false">IF(M18="Y",O18,H18)&amp;""</f>
         <v>CL21A106KAFN3NE</v>
       </c>
       <c r="X18" s="8" t="str">
-        <f aca="false">IF(M18="Y",P18,I18)</f>
+        <f aca="false">IF(M18="Y",P18,I18)&amp;""</f>
         <v>1276-2890-1-ND</v>
       </c>
       <c r="Y18" s="12" t="n">
@@ -2750,7 +2734,7 @@
         <v>0.632</v>
       </c>
       <c r="Z18" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AA18" s="8" t="str">
         <f aca="false">IF(W18="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W18,"open"))</f>
@@ -2762,16 +2746,16 @@
         <v>12</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>49</v>
@@ -2780,10 +2764,10 @@
         <v>50</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J19" s="14" t="n">
         <v>390169</v>
@@ -2813,15 +2797,15 @@
         <v>6</v>
       </c>
       <c r="V19" s="13" t="str">
-        <f aca="false">IF(M19="Y",N19,G19)</f>
+        <f aca="false">IF(M19="Y",N19,G19)&amp;""</f>
         <v>Samsung Electro-Mechanics</v>
       </c>
       <c r="W19" s="13" t="str">
-        <f aca="false">IF(M19="Y",O19,H19)</f>
+        <f aca="false">IF(M19="Y",O19,H19)&amp;""</f>
         <v>CL21B225KAFNNNE</v>
       </c>
       <c r="X19" s="13" t="str">
-        <f aca="false">IF(M19="Y",P19,I19)</f>
+        <f aca="false">IF(M19="Y",P19,I19)&amp;""</f>
         <v>1276-2954-1-ND</v>
       </c>
       <c r="Y19" s="16" t="n">
@@ -2839,28 +2823,28 @@
         <v>13</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G20" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="I20" s="8" t="s">
         <v>129</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>131</v>
       </c>
       <c r="J20" s="9" t="n">
         <v>436448</v>
@@ -2890,15 +2874,15 @@
         <v>3</v>
       </c>
       <c r="V20" s="8" t="str">
-        <f aca="false">IF(M20="Y",N20,G20)</f>
+        <f aca="false">IF(M20="Y",N20,G20)&amp;""</f>
         <v>Lite-On Inc.</v>
       </c>
       <c r="W20" s="8" t="str">
-        <f aca="false">IF(M20="Y",O20,H20)</f>
+        <f aca="false">IF(M20="Y",O20,H20)&amp;""</f>
         <v>LTST-C170KRKT</v>
       </c>
       <c r="X20" s="8" t="str">
-        <f aca="false">IF(M20="Y",P20,I20)</f>
+        <f aca="false">IF(M20="Y",P20,I20)&amp;""</f>
         <v>160-1415-1-ND</v>
       </c>
       <c r="Y20" s="12" t="n">
@@ -2906,7 +2890,7 @@
         <v>0.54</v>
       </c>
       <c r="Z20" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="AA20" s="8" t="str">
         <f aca="false">IF(W20="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W20,"open"))</f>
@@ -2918,28 +2902,28 @@
         <v>14</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>49</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J21" s="14" t="n">
         <v>477688</v>
@@ -2969,15 +2953,15 @@
         <v>4</v>
       </c>
       <c r="V21" s="13" t="str">
-        <f aca="false">IF(M21="Y",N21,G21)</f>
+        <f aca="false">IF(M21="Y",N21,G21)&amp;""</f>
         <v>Lite-On Inc.</v>
       </c>
       <c r="W21" s="13" t="str">
-        <f aca="false">IF(M21="Y",O21,H21)</f>
+        <f aca="false">IF(M21="Y",O21,H21)&amp;""</f>
         <v>LTST-C170KGKT</v>
       </c>
       <c r="X21" s="13" t="str">
-        <f aca="false">IF(M21="Y",P21,I21)</f>
+        <f aca="false">IF(M21="Y",P21,I21)&amp;""</f>
         <v>160-1414-1-ND</v>
       </c>
       <c r="Y21" s="16" t="n">
@@ -2995,28 +2979,28 @@
         <v>15</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="F22" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="G22" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="H22" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="I22" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>144</v>
       </c>
       <c r="J22" s="9" t="n">
         <v>141918</v>
@@ -3046,15 +3030,15 @@
         <v>1</v>
       </c>
       <c r="V22" s="8" t="str">
-        <f aca="false">IF(M22="Y",N22,G22)</f>
+        <f aca="false">IF(M22="Y",N22,G22)&amp;""</f>
         <v>Vishay General Semiconductor</v>
       </c>
       <c r="W22" s="8" t="str">
-        <f aca="false">IF(M22="Y",O22,H22)</f>
+        <f aca="false">IF(M22="Y",O22,H22)&amp;""</f>
         <v>SS14-E3/61T</v>
       </c>
       <c r="X22" s="8" t="str">
-        <f aca="false">IF(M22="Y",P22,I22)</f>
+        <f aca="false">IF(M22="Y",P22,I22)&amp;""</f>
         <v>SS14-E3/61TGICT-ND</v>
       </c>
       <c r="Y22" s="12" t="n">
@@ -3072,28 +3056,28 @@
         <v>16</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D23" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="F23" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="G23" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="H23" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="I23" s="13" t="s">
         <v>149</v>
-      </c>
-      <c r="H23" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="I23" s="13" t="s">
-        <v>151</v>
       </c>
       <c r="J23" s="14" t="n">
         <v>1148672</v>
@@ -3123,15 +3107,15 @@
         <v>4</v>
       </c>
       <c r="V23" s="13" t="str">
-        <f aca="false">IF(M23="Y",N23,G23)</f>
+        <f aca="false">IF(M23="Y",N23,G23)&amp;""</f>
         <v>Murata Electronics</v>
       </c>
       <c r="W23" s="13" t="str">
-        <f aca="false">IF(M23="Y",O23,H23)</f>
+        <f aca="false">IF(M23="Y",O23,H23)&amp;""</f>
         <v>BLM15AG601SN1D</v>
       </c>
       <c r="X23" s="13" t="str">
-        <f aca="false">IF(M23="Y",P23,I23)</f>
+        <f aca="false">IF(M23="Y",P23,I23)&amp;""</f>
         <v>490-1006-1-ND</v>
       </c>
       <c r="Y23" s="16" t="n">
@@ -3149,28 +3133,28 @@
         <v>17</v>
       </c>
       <c r="B24" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="F24" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="G24" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="H24" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="I24" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>158</v>
       </c>
       <c r="J24" s="9" t="n">
         <v>145796</v>
@@ -3200,15 +3184,15 @@
         <v>1</v>
       </c>
       <c r="V24" s="8" t="str">
-        <f aca="false">IF(M24="Y",N24,G24)</f>
+        <f aca="false">IF(M24="Y",N24,G24)&amp;""</f>
         <v>GCT</v>
       </c>
       <c r="W24" s="8" t="str">
-        <f aca="false">IF(M24="Y",O24,H24)</f>
+        <f aca="false">IF(M24="Y",O24,H24)&amp;""</f>
         <v>USB4110-GF-A</v>
       </c>
       <c r="X24" s="8" t="str">
-        <f aca="false">IF(M24="Y",P24,I24)</f>
+        <f aca="false">IF(M24="Y",P24,I24)&amp;""</f>
         <v>2073-USB4110-GF-A-1-ND</v>
       </c>
       <c r="Y24" s="12" t="n">
@@ -3226,28 +3210,28 @@
         <v>18</v>
       </c>
       <c r="B25" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="E25" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="C25" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="F25" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="G25" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="H25" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="G25" s="13" t="s">
+      <c r="I25" s="13" t="s">
         <v>163</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="I25" s="13" t="s">
-        <v>165</v>
       </c>
       <c r="J25" s="14" t="n">
         <v>12098</v>
@@ -3277,15 +3261,15 @@
         <v>1</v>
       </c>
       <c r="V25" s="13" t="str">
-        <f aca="false">IF(M25="Y",N25,G25)</f>
+        <f aca="false">IF(M25="Y",N25,G25)&amp;""</f>
         <v>JST Sales America Inc.</v>
       </c>
       <c r="W25" s="13" t="str">
-        <f aca="false">IF(M25="Y",O25,H25)</f>
+        <f aca="false">IF(M25="Y",O25,H25)&amp;""</f>
         <v>B02B-XASK-1</v>
       </c>
       <c r="X25" s="13" t="str">
-        <f aca="false">IF(M25="Y",P25,I25)</f>
+        <f aca="false">IF(M25="Y",P25,I25)&amp;""</f>
         <v>455-B02B-XASK-1-ND</v>
       </c>
       <c r="Y25" s="16" t="n">
@@ -3293,7 +3277,7 @@
         <v>0.16</v>
       </c>
       <c r="Z25" s="13" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AA25" s="13" t="str">
         <f aca="false">IF(W25="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W25,"open"))</f>
@@ -3305,28 +3289,28 @@
         <v>19</v>
       </c>
       <c r="B26" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="C26" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="F26" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="G26" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="H26" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="I26" s="8" t="s">
         <v>171</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="J26" s="9" t="n">
         <v>42330</v>
@@ -3356,15 +3340,15 @@
         <v>1</v>
       </c>
       <c r="V26" s="8" t="str">
-        <f aca="false">IF(M26="Y",N26,G26)</f>
+        <f aca="false">IF(M26="Y",N26,G26)&amp;""</f>
         <v>Sullins Connector Solutions</v>
       </c>
       <c r="W26" s="8" t="str">
-        <f aca="false">IF(M26="Y",O26,H26)</f>
+        <f aca="false">IF(M26="Y",O26,H26)&amp;""</f>
         <v>PREC004SAAN-RC</v>
       </c>
       <c r="X26" s="8" t="str">
-        <f aca="false">IF(M26="Y",P26,I26)</f>
+        <f aca="false">IF(M26="Y",P26,I26)&amp;""</f>
         <v>35-PREC004SAAN-RC-ND</v>
       </c>
       <c r="Y26" s="12" t="n">
@@ -3382,28 +3366,28 @@
         <v>20</v>
       </c>
       <c r="B27" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="C27" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="13" t="s">
+      <c r="F27" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="G27" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="H27" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="F27" s="13" t="s">
+      <c r="I27" s="13" t="s">
         <v>177</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="H27" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>179</v>
       </c>
       <c r="J27" s="14" t="n">
         <v>55276</v>
@@ -3433,15 +3417,15 @@
         <v>1</v>
       </c>
       <c r="V27" s="13" t="str">
-        <f aca="false">IF(M27="Y",N27,G27)</f>
+        <f aca="false">IF(M27="Y",N27,G27)&amp;""</f>
         <v>Sullins Connector Solutions</v>
       </c>
       <c r="W27" s="13" t="str">
-        <f aca="false">IF(M27="Y",O27,H27)</f>
+        <f aca="false">IF(M27="Y",O27,H27)&amp;""</f>
         <v>PREC002SAAN-RC</v>
       </c>
       <c r="X27" s="13" t="str">
-        <f aca="false">IF(M27="Y",P27,I27)</f>
+        <f aca="false">IF(M27="Y",P27,I27)&amp;""</f>
         <v>35-PREC002SAAN-RC-ND</v>
       </c>
       <c r="Y27" s="16" t="n">
@@ -3449,7 +3433,7 @@
         <v>0.1</v>
       </c>
       <c r="Z27" s="13" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AA27" s="13" t="str">
         <f aca="false">IF(W27="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W27,"open"))</f>
@@ -3461,19 +3445,19 @@
         <v>21</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D28" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>182</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>184</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
@@ -3499,24 +3483,24 @@
         <f aca="false">IF(S28="Y",C28*$B$4+T28,0)</f>
         <v>0</v>
       </c>
-      <c r="V28" s="8" t="n">
-        <f aca="false">IF(M28="Y",N28,G28)</f>
-        <v>0</v>
-      </c>
-      <c r="W28" s="8" t="n">
-        <f aca="false">IF(M28="Y",O28,H28)</f>
-        <v>0</v>
-      </c>
-      <c r="X28" s="8" t="n">
-        <f aca="false">IF(M28="Y",P28,I28)</f>
-        <v>0</v>
+      <c r="V28" s="8" t="str">
+        <f aca="false">IF(M28="Y",N28,G28)&amp;""</f>
+        <v/>
+      </c>
+      <c r="W28" s="8" t="str">
+        <f aca="false">IF(M28="Y",O28,H28)&amp;""</f>
+        <v/>
+      </c>
+      <c r="X28" s="8" t="str">
+        <f aca="false">IF(M28="Y",P28,I28)&amp;""</f>
+        <v/>
       </c>
       <c r="Y28" s="12" t="n">
         <f aca="false">U28*IF(M28="Y",R28,K28)</f>
         <v>0</v>
       </c>
       <c r="Z28" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="AA28" s="8" t="str">
         <f aca="false">IF(W28="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W28,"open"))</f>
@@ -3528,28 +3512,28 @@
         <v>22</v>
       </c>
       <c r="B29" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="E29" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="13" t="s">
+      <c r="F29" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="G29" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="H29" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="I29" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="H29" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="I29" s="13" t="s">
-        <v>191</v>
       </c>
       <c r="J29" s="14" t="n">
         <v>29560</v>
@@ -3579,15 +3563,15 @@
         <v>1</v>
       </c>
       <c r="V29" s="13" t="str">
-        <f aca="false">IF(M29="Y",N29,G29)</f>
+        <f aca="false">IF(M29="Y",N29,G29)&amp;""</f>
         <v>Sullins Connector Solutions</v>
       </c>
       <c r="W29" s="13" t="str">
-        <f aca="false">IF(M29="Y",O29,H29)</f>
+        <f aca="false">IF(M29="Y",O29,H29)&amp;""</f>
         <v>PPTC081LFBN-RC</v>
       </c>
       <c r="X29" s="13" t="str">
-        <f aca="false">IF(M29="Y",P29,I29)</f>
+        <f aca="false">IF(M29="Y",P29,I29)&amp;""</f>
         <v>S7006-ND</v>
       </c>
       <c r="Y29" s="16" t="n">
@@ -3595,7 +3579,7 @@
         <v>0.58</v>
       </c>
       <c r="Z29" s="13" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="AA29" s="13" t="str">
         <f aca="false">IF(W29="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W29,"open"))</f>
@@ -3607,28 +3591,28 @@
         <v>23</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C30" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G30" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="I30" s="8" t="s">
         <v>196</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>198</v>
       </c>
       <c r="J30" s="9" t="n">
         <v>10591</v>
@@ -3658,15 +3642,15 @@
         <v>2</v>
       </c>
       <c r="V30" s="8" t="str">
-        <f aca="false">IF(M30="Y",N30,G30)</f>
+        <f aca="false">IF(M30="Y",N30,G30)&amp;""</f>
         <v>Coilcraft</v>
       </c>
       <c r="W30" s="8" t="str">
-        <f aca="false">IF(M30="Y",O30,H30)</f>
+        <f aca="false">IF(M30="Y",O30,H30)&amp;""</f>
         <v>0805CS-471XJRC</v>
       </c>
       <c r="X30" s="8" t="str">
-        <f aca="false">IF(M30="Y",P30,I30)</f>
+        <f aca="false">IF(M30="Y",P30,I30)&amp;""</f>
         <v>2457-0805CS-471XJRC-ND</v>
       </c>
       <c r="Y30" s="12" t="n">
@@ -3674,7 +3658,7 @@
         <v>2.68</v>
       </c>
       <c r="Z30" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AA30" s="8" t="str">
         <f aca="false">IF(W30="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W30,"open"))</f>
@@ -3686,28 +3670,28 @@
         <v>24</v>
       </c>
       <c r="B31" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="E31" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="C31" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="13" t="s">
+      <c r="F31" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="G31" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="H31" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="I31" s="13" t="s">
         <v>203</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="I31" s="13" t="s">
-        <v>205</v>
       </c>
       <c r="J31" s="14" t="n">
         <v>303749</v>
@@ -3737,15 +3721,15 @@
         <v>1</v>
       </c>
       <c r="V31" s="13" t="str">
-        <f aca="false">IF(M31="Y",N31,G31)</f>
+        <f aca="false">IF(M31="Y",N31,G31)&amp;""</f>
         <v>Alpha &amp; Omega Semiconductor</v>
       </c>
       <c r="W31" s="13" t="str">
-        <f aca="false">IF(M31="Y",O31,H31)</f>
+        <f aca="false">IF(M31="Y",O31,H31)&amp;""</f>
         <v>AO3400A</v>
       </c>
       <c r="X31" s="13" t="str">
-        <f aca="false">IF(M31="Y",P31,I31)</f>
+        <f aca="false">IF(M31="Y",P31,I31)&amp;""</f>
         <v>785-1000-1-ND</v>
       </c>
       <c r="Y31" s="16" t="n">
@@ -3763,28 +3747,28 @@
         <v>25</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C32" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G32" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="I32" s="8" t="s">
         <v>209</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="I32" s="8" t="s">
-        <v>211</v>
       </c>
       <c r="J32" s="9" t="n">
         <v>101761</v>
@@ -3814,15 +3798,15 @@
         <v>4</v>
       </c>
       <c r="V32" s="8" t="str">
-        <f aca="false">IF(M32="Y",N32,G32)</f>
+        <f aca="false">IF(M32="Y",N32,G32)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W32" s="8" t="str">
-        <f aca="false">IF(M32="Y",O32,H32)</f>
+        <f aca="false">IF(M32="Y",O32,H32)&amp;""</f>
         <v>RMCF0805FT5K10</v>
       </c>
       <c r="X32" s="8" t="str">
-        <f aca="false">IF(M32="Y",P32,I32)</f>
+        <f aca="false">IF(M32="Y",P32,I32)&amp;""</f>
         <v>RMCF0805FT5K10CT-ND</v>
       </c>
       <c r="Y32" s="12" t="n">
@@ -3830,7 +3814,7 @@
         <v>0.108</v>
       </c>
       <c r="Z32" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="AA32" s="8" t="str">
         <f aca="false">IF(W32="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W32,"open"))</f>
@@ -3842,28 +3826,28 @@
         <v>26</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>5</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F33" s="13" t="s">
         <v>49</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="J33" s="14" t="n">
         <v>106645</v>
@@ -3893,15 +3877,15 @@
         <v>7</v>
       </c>
       <c r="V33" s="13" t="str">
-        <f aca="false">IF(M33="Y",N33,G33)</f>
+        <f aca="false">IF(M33="Y",N33,G33)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W33" s="13" t="str">
-        <f aca="false">IF(M33="Y",O33,H33)</f>
+        <f aca="false">IF(M33="Y",O33,H33)&amp;""</f>
         <v>RMCF0805FT470R</v>
       </c>
       <c r="X33" s="13" t="str">
-        <f aca="false">IF(M33="Y",P33,I33)</f>
+        <f aca="false">IF(M33="Y",P33,I33)&amp;""</f>
         <v>RMCF0805FT470RCT-ND</v>
       </c>
       <c r="Y33" s="16" t="n">
@@ -3919,28 +3903,28 @@
         <v>27</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>218</v>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>220</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J34" s="9" t="n">
         <v>320655</v>
@@ -3955,13 +3939,13 @@
         <v>53</v>
       </c>
       <c r="N34" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O34" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="P34" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="Q34" s="9" t="n">
         <v>119534</v>
@@ -3980,15 +3964,15 @@
         <v>3</v>
       </c>
       <c r="V34" s="8" t="str">
-        <f aca="false">IF(M34="Y",N34,G34)</f>
+        <f aca="false">IF(M34="Y",N34,G34)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W34" s="8" t="str">
-        <f aca="false">IF(M34="Y",O34,H34)</f>
+        <f aca="false">IF(M34="Y",O34,H34)&amp;""</f>
         <v>RMCF0805FT1K00</v>
       </c>
       <c r="X34" s="8" t="str">
-        <f aca="false">IF(M34="Y",P34,I34)</f>
+        <f aca="false">IF(M34="Y",P34,I34)&amp;""</f>
         <v>RMCF0805FT1K00CT-ND</v>
       </c>
       <c r="Y34" s="12" t="n">
@@ -3996,7 +3980,7 @@
         <v>0.081</v>
       </c>
       <c r="Z34" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="AA34" s="8" t="str">
         <f aca="false">IF(W34="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W34,"open"))</f>
@@ -4008,28 +3992,28 @@
         <v>28</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>5</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F35" s="13" t="s">
         <v>49</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="J35" s="14" t="n">
         <v>3852513</v>
@@ -4059,15 +4043,15 @@
         <v>7</v>
       </c>
       <c r="V35" s="13" t="str">
-        <f aca="false">IF(M35="Y",N35,G35)</f>
+        <f aca="false">IF(M35="Y",N35,G35)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W35" s="13" t="str">
-        <f aca="false">IF(M35="Y",O35,H35)</f>
+        <f aca="false">IF(M35="Y",O35,H35)&amp;""</f>
         <v>RMCF0805FT10K0</v>
       </c>
       <c r="X35" s="13" t="str">
-        <f aca="false">IF(M35="Y",P35,I35)</f>
+        <f aca="false">IF(M35="Y",P35,I35)&amp;""</f>
         <v>RMCF0805FT10K0CT-ND</v>
       </c>
       <c r="Y35" s="16" t="n">
@@ -4085,28 +4069,28 @@
         <v>29</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="E36" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>233</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="J36" s="9" t="n">
         <v>149568</v>
@@ -4136,15 +4120,15 @@
         <v>3</v>
       </c>
       <c r="V36" s="8" t="str">
-        <f aca="false">IF(M36="Y",N36,G36)</f>
+        <f aca="false">IF(M36="Y",N36,G36)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W36" s="8" t="str">
-        <f aca="false">IF(M36="Y",O36,H36)</f>
+        <f aca="false">IF(M36="Y",O36,H36)&amp;""</f>
         <v>RMCF0805FT1K50</v>
       </c>
       <c r="X36" s="8" t="str">
-        <f aca="false">IF(M36="Y",P36,I36)</f>
+        <f aca="false">IF(M36="Y",P36,I36)&amp;""</f>
         <v>RMCF0805FT1K50CT-ND</v>
       </c>
       <c r="Y36" s="12" t="n">
@@ -4152,7 +4136,7 @@
         <v>0.081</v>
       </c>
       <c r="Z36" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="AA36" s="8" t="str">
         <f aca="false">IF(W36="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W36,"open"))</f>
@@ -4164,28 +4148,28 @@
         <v>30</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>3</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F37" s="13" t="s">
         <v>49</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J37" s="14" t="n">
         <v>12637</v>
@@ -4215,15 +4199,15 @@
         <v>5</v>
       </c>
       <c r="V37" s="13" t="str">
-        <f aca="false">IF(M37="Y",N37,G37)</f>
+        <f aca="false">IF(M37="Y",N37,G37)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W37" s="13" t="str">
-        <f aca="false">IF(M37="Y",O37,H37)</f>
+        <f aca="false">IF(M37="Y",O37,H37)&amp;""</f>
         <v>RMCF0805FT4M70</v>
       </c>
       <c r="X37" s="13" t="str">
-        <f aca="false">IF(M37="Y",P37,I37)</f>
+        <f aca="false">IF(M37="Y",P37,I37)&amp;""</f>
         <v>RMCF0805FT4M70CT-ND</v>
       </c>
       <c r="Y37" s="16" t="n">
@@ -4241,28 +4225,28 @@
         <v>31</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>242</v>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>244</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>49</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J38" s="9" t="n">
         <v>6211</v>
@@ -4292,15 +4276,15 @@
         <v>3</v>
       </c>
       <c r="V38" s="8" t="str">
-        <f aca="false">IF(M38="Y",N38,G38)</f>
+        <f aca="false">IF(M38="Y",N38,G38)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W38" s="8" t="str">
-        <f aca="false">IF(M38="Y",O38,H38)</f>
+        <f aca="false">IF(M38="Y",O38,H38)&amp;""</f>
         <v>RMCF0805FT2M70</v>
       </c>
       <c r="X38" s="8" t="str">
-        <f aca="false">IF(M38="Y",P38,I38)</f>
+        <f aca="false">IF(M38="Y",P38,I38)&amp;""</f>
         <v>RMCF0805FT2M70CT-ND</v>
       </c>
       <c r="Y38" s="12" t="n">
@@ -4318,28 +4302,28 @@
         <v>32</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F39" s="13" t="s">
         <v>49</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="I39" s="13" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="J39" s="14" t="n">
         <v>3287189</v>
@@ -4369,15 +4353,15 @@
         <v>4</v>
       </c>
       <c r="V39" s="13" t="str">
-        <f aca="false">IF(M39="Y",N39,G39)</f>
+        <f aca="false">IF(M39="Y",N39,G39)&amp;""</f>
         <v>Stackpole Electronics</v>
       </c>
       <c r="W39" s="13" t="str">
-        <f aca="false">IF(M39="Y",O39,H39)</f>
+        <f aca="false">IF(M39="Y",O39,H39)&amp;""</f>
         <v>RMCF0805ZT0R00</v>
       </c>
       <c r="X39" s="13" t="str">
-        <f aca="false">IF(M39="Y",P39,I39)</f>
+        <f aca="false">IF(M39="Y",P39,I39)&amp;""</f>
         <v>RMCF0805ZT0R00CT-ND</v>
       </c>
       <c r="Y39" s="16" t="n">
@@ -4395,28 +4379,28 @@
         <v>33</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C40" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D40" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="F40" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="G40" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="H40" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="I40" s="8" t="s">
         <v>256</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="I40" s="8" t="s">
-        <v>258</v>
       </c>
       <c r="J40" s="9" t="n">
         <v>20227</v>
@@ -4446,15 +4430,15 @@
         <v>3</v>
       </c>
       <c r="V40" s="8" t="str">
-        <f aca="false">IF(M40="Y",N40,G40)</f>
+        <f aca="false">IF(M40="Y",N40,G40)&amp;""</f>
         <v>C&amp;K</v>
       </c>
       <c r="W40" s="8" t="str">
-        <f aca="false">IF(M40="Y",O40,H40)</f>
+        <f aca="false">IF(M40="Y",O40,H40)&amp;""</f>
         <v>PTS636SM25SMTR LFS</v>
       </c>
       <c r="X40" s="8" t="str">
-        <f aca="false">IF(M40="Y",P40,I40)</f>
+        <f aca="false">IF(M40="Y",P40,I40)&amp;""</f>
         <v>CKN12321-1-ND</v>
       </c>
       <c r="Y40" s="12" t="n">
@@ -4462,7 +4446,7 @@
         <v>0.87</v>
       </c>
       <c r="Z40" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AA40" s="8" t="str">
         <f aca="false">IF(W40="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W40,"open"))</f>
@@ -4474,28 +4458,28 @@
         <v>34</v>
       </c>
       <c r="B41" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="E41" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="C41" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="13" t="s">
+      <c r="F41" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="G41" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="F41" s="13" t="s">
+      <c r="H41" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="G41" s="13" t="s">
+      <c r="I41" s="13" t="s">
         <v>264</v>
-      </c>
-      <c r="H41" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="I41" s="13" t="s">
-        <v>266</v>
       </c>
       <c r="J41" s="14" t="n">
         <v>10220</v>
@@ -4525,15 +4509,15 @@
         <v>1</v>
       </c>
       <c r="V41" s="13" t="str">
-        <f aca="false">IF(M41="Y",N41,G41)</f>
+        <f aca="false">IF(M41="Y",N41,G41)&amp;""</f>
         <v>Vishay BC Components</v>
       </c>
       <c r="W41" s="13" t="str">
-        <f aca="false">IF(M41="Y",O41,H41)</f>
+        <f aca="false">IF(M41="Y",O41,H41)&amp;""</f>
         <v>NTCLE100E3103JB0</v>
       </c>
       <c r="X41" s="13" t="str">
-        <f aca="false">IF(M41="Y",P41,I41)</f>
+        <f aca="false">IF(M41="Y",P41,I41)&amp;""</f>
         <v>BC2301-ND</v>
       </c>
       <c r="Y41" s="16" t="n">
@@ -4541,7 +4525,7 @@
         <v>0.6</v>
       </c>
       <c r="Z41" s="13" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AA41" s="13" t="str">
         <f aca="false">IF(W41="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W41,"open"))</f>
@@ -4553,28 +4537,28 @@
         <v>35</v>
       </c>
       <c r="B42" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="E42" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="C42" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="8" t="s">
+      <c r="F42" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="G42" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="F42" s="8" t="s">
+      <c r="H42" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="G42" s="8" t="s">
+      <c r="I42" s="8" t="s">
         <v>272</v>
-      </c>
-      <c r="H42" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>274</v>
       </c>
       <c r="J42" s="9" t="n">
         <v>1307</v>
@@ -4604,15 +4588,15 @@
         <v>1</v>
       </c>
       <c r="V42" s="8" t="str">
-        <f aca="false">IF(M42="Y",N42,G42)</f>
+        <f aca="false">IF(M42="Y",N42,G42)&amp;""</f>
         <v>STMicroelectronics</v>
       </c>
       <c r="W42" s="8" t="str">
-        <f aca="false">IF(M42="Y",O42,H42)</f>
+        <f aca="false">IF(M42="Y",O42,H42)&amp;""</f>
         <v>STM32L432KCU6TR</v>
       </c>
       <c r="X42" s="8" t="str">
-        <f aca="false">IF(M42="Y",P42,I42)</f>
+        <f aca="false">IF(M42="Y",P42,I42)&amp;""</f>
         <v>497-STM32L432KCU6TRCT-ND</v>
       </c>
       <c r="Y42" s="12" t="n">
@@ -4620,7 +4604,7 @@
         <v>6.1</v>
       </c>
       <c r="Z42" s="8" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AA42" s="8" t="str">
         <f aca="false">IF(W42="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W42,"open"))</f>
@@ -4632,28 +4616,28 @@
         <v>36</v>
       </c>
       <c r="B43" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="E43" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="C43" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="13" t="s">
+      <c r="F43" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="G43" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="F43" s="13" t="s">
+      <c r="H43" s="13" t="s">
         <v>279</v>
       </c>
-      <c r="G43" s="13" t="s">
+      <c r="I43" s="13" t="s">
         <v>280</v>
-      </c>
-      <c r="H43" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="I43" s="13" t="s">
-        <v>282</v>
       </c>
       <c r="J43" s="14" t="n">
         <v>1437</v>
@@ -4683,15 +4667,15 @@
         <v>1</v>
       </c>
       <c r="V43" s="13" t="str">
-        <f aca="false">IF(M43="Y",N43,G43)</f>
+        <f aca="false">IF(M43="Y",N43,G43)&amp;""</f>
         <v>Microchip Technology</v>
       </c>
       <c r="W43" s="13" t="str">
-        <f aca="false">IF(M43="Y",O43,H43)</f>
+        <f aca="false">IF(M43="Y",O43,H43)&amp;""</f>
         <v>MCP73833-AMI/UN</v>
       </c>
       <c r="X43" s="13" t="str">
-        <f aca="false">IF(M43="Y",P43,I43)</f>
+        <f aca="false">IF(M43="Y",P43,I43)&amp;""</f>
         <v>MCP73833-AMI/UN-ND</v>
       </c>
       <c r="Y43" s="16" t="n">
@@ -4699,7 +4683,7 @@
         <v>1.14</v>
       </c>
       <c r="Z43" s="13" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="AA43" s="13" t="str">
         <f aca="false">IF(W43="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W43,"open"))</f>
@@ -4711,28 +4695,28 @@
         <v>37</v>
       </c>
       <c r="B44" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="C44" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="8" t="s">
+      <c r="F44" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="G44" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="H44" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="G44" s="8" t="s">
+      <c r="I44" s="8" t="s">
         <v>288</v>
-      </c>
-      <c r="H44" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>290</v>
       </c>
       <c r="J44" s="9" t="n">
         <v>6864</v>
@@ -4762,15 +4746,15 @@
         <v>1</v>
       </c>
       <c r="V44" s="8" t="str">
-        <f aca="false">IF(M44="Y",N44,G44)</f>
+        <f aca="false">IF(M44="Y",N44,G44)&amp;""</f>
         <v>Texas Instruments</v>
       </c>
       <c r="W44" s="8" t="str">
-        <f aca="false">IF(M44="Y",O44,H44)</f>
+        <f aca="false">IF(M44="Y",O44,H44)&amp;""</f>
         <v>TPS7A0233PDBVR</v>
       </c>
       <c r="X44" s="8" t="str">
-        <f aca="false">IF(M44="Y",P44,I44)</f>
+        <f aca="false">IF(M44="Y",P44,I44)&amp;""</f>
         <v>296-TPS7A0233PDBVRCT-ND</v>
       </c>
       <c r="Y44" s="12" t="n">
@@ -4788,28 +4772,28 @@
         <v>38</v>
       </c>
       <c r="B45" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="E45" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="C45" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="13" t="s">
+      <c r="F45" s="13" t="s">
         <v>292</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="G45" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="H45" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="F45" s="13" t="s">
+      <c r="I45" s="13" t="s">
         <v>294</v>
-      </c>
-      <c r="G45" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="H45" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="I45" s="13" t="s">
-        <v>296</v>
       </c>
       <c r="J45" s="14" t="n">
         <v>0</v>
@@ -4824,13 +4808,13 @@
         <v>53</v>
       </c>
       <c r="N45" s="13" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="O45" s="13" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="P45" s="13" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="Q45" s="14" t="n">
         <v>4278</v>
@@ -4849,15 +4833,15 @@
         <v>1</v>
       </c>
       <c r="V45" s="13" t="str">
-        <f aca="false">IF(M45="Y",N45,G45)</f>
+        <f aca="false">IF(M45="Y",N45,G45)&amp;""</f>
         <v>STMicroelectronics</v>
       </c>
       <c r="W45" s="13" t="str">
-        <f aca="false">IF(M45="Y",O45,H45)</f>
+        <f aca="false">IF(M45="Y",O45,H45)&amp;""</f>
         <v>ST25R3916-AQWT</v>
       </c>
       <c r="X45" s="13" t="str">
-        <f aca="false">IF(M45="Y",P45,I45)</f>
+        <f aca="false">IF(M45="Y",P45,I45)&amp;""</f>
         <v>497-18366-1-ND</v>
       </c>
       <c r="Y45" s="16" t="n">
@@ -4865,7 +4849,7 @@
         <v>6.51</v>
       </c>
       <c r="Z45" s="13" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AA45" s="13" t="str">
         <f aca="false">IF(W45="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W45,"open"))</f>
@@ -4877,28 +4861,28 @@
         <v>39</v>
       </c>
       <c r="B46" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="E46" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="C46" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="8" t="s">
+      <c r="F46" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="G46" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="F46" s="8" t="s">
+      <c r="I46" s="8" t="s">
         <v>303</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>304</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>305</v>
       </c>
       <c r="J46" s="9" t="n">
         <v>39458</v>
@@ -4928,15 +4912,15 @@
         <v>1</v>
       </c>
       <c r="V46" s="8" t="str">
-        <f aca="false">IF(M46="Y",N46,G46)</f>
+        <f aca="false">IF(M46="Y",N46,G46)&amp;""</f>
         <v>STMicroelectronics</v>
       </c>
       <c r="W46" s="8" t="str">
-        <f aca="false">IF(M46="Y",O46,H46)</f>
+        <f aca="false">IF(M46="Y",O46,H46)&amp;""</f>
         <v>USBLC6-2SC6Y</v>
       </c>
       <c r="X46" s="8" t="str">
-        <f aca="false">IF(M46="Y",P46,I46)</f>
+        <f aca="false">IF(M46="Y",P46,I46)&amp;""</f>
         <v>497-11882-1-ND</v>
       </c>
       <c r="Y46" s="12" t="n">
@@ -4944,7 +4928,7 @@
         <v>0.71</v>
       </c>
       <c r="Z46" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="AA46" s="8" t="str">
         <f aca="false">IF(W46="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W46,"open"))</f>
@@ -4956,28 +4940,28 @@
         <v>40</v>
       </c>
       <c r="B47" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="E47" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="C47" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="13" t="s">
+      <c r="F47" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="G47" s="13" t="s">
         <v>309</v>
       </c>
-      <c r="F47" s="13" t="s">
+      <c r="H47" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="G47" s="13" t="s">
+      <c r="I47" s="13" t="s">
         <v>311</v>
-      </c>
-      <c r="H47" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="I47" s="13" t="s">
-        <v>313</v>
       </c>
       <c r="J47" s="14" t="n">
         <v>15659</v>
@@ -5007,15 +4991,15 @@
         <v>1</v>
       </c>
       <c r="V47" s="13" t="str">
-        <f aca="false">IF(M47="Y",N47,G47)</f>
+        <f aca="false">IF(M47="Y",N47,G47)&amp;""</f>
         <v>Abracon LLC</v>
       </c>
       <c r="W47" s="13" t="str">
-        <f aca="false">IF(M47="Y",O47,H47)</f>
+        <f aca="false">IF(M47="Y",O47,H47)&amp;""</f>
         <v>ABM8-27.120MHZ-10-D1G-T</v>
       </c>
       <c r="X47" s="13" t="str">
-        <f aca="false">IF(M47="Y",P47,I47)</f>
+        <f aca="false">IF(M47="Y",P47,I47)&amp;""</f>
         <v>535-14403-1-ND</v>
       </c>
       <c r="Y47" s="16" t="n">
@@ -5023,7 +5007,7 @@
         <v>0.46</v>
       </c>
       <c r="Z47" s="13" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="AA47" s="13" t="str">
         <f aca="false">IF(W47="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W47,"open"))</f>
@@ -5035,28 +5019,28 @@
         <v>41</v>
       </c>
       <c r="B48" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="C48" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="E48" s="8" t="s">
         <v>315</v>
       </c>
-      <c r="C48" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="8" t="s">
+      <c r="F48" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="E48" s="8" t="s">
+      <c r="G48" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="H48" s="8" t="s">
         <v>317</v>
       </c>
-      <c r="F48" s="8" t="s">
+      <c r="I48" s="8" t="s">
         <v>318</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>311</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>319</v>
-      </c>
-      <c r="I48" s="8" t="s">
-        <v>320</v>
       </c>
       <c r="J48" s="9" t="n">
         <v>52806</v>
@@ -5086,15 +5070,15 @@
         <v>1</v>
       </c>
       <c r="V48" s="8" t="str">
-        <f aca="false">IF(M48="Y",N48,G48)</f>
+        <f aca="false">IF(M48="Y",N48,G48)&amp;""</f>
         <v>Abracon LLC</v>
       </c>
       <c r="W48" s="8" t="str">
-        <f aca="false">IF(M48="Y",O48,H48)</f>
+        <f aca="false">IF(M48="Y",O48,H48)&amp;""</f>
         <v>ABS07-120-32.768KHZ-T</v>
       </c>
       <c r="X48" s="8" t="str">
-        <f aca="false">IF(M48="Y",P48,I48)</f>
+        <f aca="false">IF(M48="Y",P48,I48)&amp;""</f>
         <v>535-11937-1-ND</v>
       </c>
       <c r="Y48" s="12" t="n">
@@ -5102,7 +5086,7 @@
         <v>0.94</v>
       </c>
       <c r="Z48" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="AA48" s="8" t="str">
         <f aca="false">IF(W48="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W48,"open"))</f>
@@ -5114,19 +5098,19 @@
         <v>42</v>
       </c>
       <c r="B49" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="E49" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="C49" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="13" t="s">
+      <c r="F49" s="13" t="s">
         <v>323</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="F49" s="13" t="s">
-        <v>325</v>
       </c>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
@@ -5152,24 +5136,24 @@
         <f aca="false">IF(S49="Y",C49*$B$4+T49,0)</f>
         <v>0</v>
       </c>
-      <c r="V49" s="13" t="n">
-        <f aca="false">IF(M49="Y",N49,G49)</f>
-        <v>0</v>
-      </c>
-      <c r="W49" s="13" t="n">
-        <f aca="false">IF(M49="Y",O49,H49)</f>
-        <v>0</v>
-      </c>
-      <c r="X49" s="13" t="n">
-        <f aca="false">IF(M49="Y",P49,I49)</f>
-        <v>0</v>
+      <c r="V49" s="13" t="str">
+        <f aca="false">IF(M49="Y",N49,G49)&amp;""</f>
+        <v/>
+      </c>
+      <c r="W49" s="13" t="str">
+        <f aca="false">IF(M49="Y",O49,H49)&amp;""</f>
+        <v/>
+      </c>
+      <c r="X49" s="13" t="str">
+        <f aca="false">IF(M49="Y",P49,I49)&amp;""</f>
+        <v/>
       </c>
       <c r="Y49" s="16" t="n">
         <f aca="false">U49*IF(M49="Y",R49,K49)</f>
         <v>0</v>
       </c>
       <c r="Z49" s="13" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AA49" s="13" t="str">
         <f aca="false">IF(W49="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W49,"open"))</f>
@@ -5181,26 +5165,26 @@
         <v>43</v>
       </c>
       <c r="B50" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E50" s="8" t="s">
         <v>327</v>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>328</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>329</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H50" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="I50" s="8" t="s">
         <v>328</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="J50" s="9" t="n">
         <v>74040</v>
@@ -5230,15 +5214,15 @@
         <v>0</v>
       </c>
       <c r="V50" s="8" t="str">
-        <f aca="false">IF(M50="Y",N50,G50)</f>
+        <f aca="false">IF(M50="Y",N50,G50)&amp;""</f>
         <v>JST Sales America Inc.</v>
       </c>
       <c r="W50" s="8" t="str">
-        <f aca="false">IF(M50="Y",O50,H50)</f>
+        <f aca="false">IF(M50="Y",O50,H50)&amp;""</f>
         <v>XAP-02V-1</v>
       </c>
       <c r="X50" s="8" t="str">
-        <f aca="false">IF(M50="Y",P50,I50)</f>
+        <f aca="false">IF(M50="Y",P50,I50)&amp;""</f>
         <v>455-1903-ND</v>
       </c>
       <c r="Y50" s="12" t="n">
@@ -5246,7 +5230,7 @@
         <v>0</v>
       </c>
       <c r="Z50" s="8" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AA50" s="8" t="str">
         <f aca="false">IF(W50="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W50,"open"))</f>
@@ -5258,26 +5242,26 @@
         <v>44</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F51" s="13"/>
       <c r="G51" s="13" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H51" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="I51" s="13" t="s">
         <v>332</v>
-      </c>
-      <c r="I51" s="13" t="s">
-        <v>334</v>
       </c>
       <c r="J51" s="14" t="n">
         <v>112000</v>
@@ -5307,15 +5291,15 @@
         <v>0</v>
       </c>
       <c r="V51" s="13" t="str">
-        <f aca="false">IF(M51="Y",N51,G51)</f>
+        <f aca="false">IF(M51="Y",N51,G51)&amp;""</f>
         <v>JST Sales America Inc.</v>
       </c>
       <c r="W51" s="13" t="str">
-        <f aca="false">IF(M51="Y",O51,H51)</f>
+        <f aca="false">IF(M51="Y",O51,H51)&amp;""</f>
         <v>SXA-001T-P0.6</v>
       </c>
       <c r="X51" s="13" t="str">
-        <f aca="false">IF(M51="Y",P51,I51)</f>
+        <f aca="false">IF(M51="Y",P51,I51)&amp;""</f>
         <v>455-1904TR-ND</v>
       </c>
       <c r="Y51" s="16" t="n">
@@ -5323,7 +5307,7 @@
         <v>0</v>
       </c>
       <c r="Z51" s="13" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="AA51" s="13" t="str">
         <f aca="false">IF(W51="","",HYPERLINK("https://www.digikey.com/en/products/result?keywords="&amp;W51,"open"))</f>
@@ -5332,19 +5316,19 @@
     </row>
     <row r="53" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="X53" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="Y53" s="17" t="n">
         <f aca="false">SUM(Y8:Y51)</f>
         <v>34.475</v>
       </c>
       <c r="Z53" s="18" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="X54" s="19" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="Y54" s="19" t="n">
         <f aca="false">COUNTIF(U8:U51,"&gt;0")</f>
@@ -5390,19 +5374,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>338</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>339</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>340</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>341</v>
       </c>
       <c r="D1" s="20" t="s">
         <v>25</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>